<commit_message>
fix: adicionado chave estrageira em animal vivo para tutor
</commit_message>
<xml_diff>
--- a/documentacao-e-dados-auxiliares/backlog.xlsx
+++ b/documentacao-e-dados-auxiliares/backlog.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Biblioteca\projetos\sistema-resgistro-analise-integrada\documentacao-e-dados-auxiliares\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26779A15-24A3-4C56-BD22-043836E25CAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083567BC-7442-443F-A159-8344CCC19DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20640" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -267,12 +267,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF38"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FF92D050"/>
         <bgColor rgb="FFFFFF00"/>
       </patternFill>
@@ -285,8 +279,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor rgb="FFFFCC00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFCC00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -304,12 +304,12 @@
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
@@ -613,30 +613,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G2" t="s">
@@ -647,16 +647,16 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
       <c r="G3" t="s">
@@ -667,16 +667,16 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" s="3" t="s">
         <v>7</v>
       </c>
       <c r="G4" t="s">
@@ -687,30 +687,30 @@
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="C5" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>12</v>
       </c>
     </row>
@@ -995,212 +995,212 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="6" t="s">
+      <c r="B27" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="C27" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="5" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="A28" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C28" t="s">
-        <v>11</v>
-      </c>
-      <c r="D28" t="s">
+      <c r="C28" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D28" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="6" t="s">
+      <c r="C29" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="3" t="s">
+      <c r="A30" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="3" t="s">
+      <c r="B30" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C30" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D30" s="3" t="s">
+      <c r="C30" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D30" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="4" t="s">
+      <c r="A31" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="4" t="s">
+      <c r="B31" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D31" s="4" t="s">
+      <c r="C31" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D31" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="4" t="s">
+      <c r="A32" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B32" s="4" t="s">
+      <c r="B32" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C32" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D32" s="4" t="s">
+      <c r="C32" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D32" s="2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B33" s="5" t="s">
+      <c r="B33" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="5" t="s">
+      <c r="C33" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A34" s="5" t="s">
+      <c r="A34" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B34" s="5" t="s">
+      <c r="B34" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D34" s="5" t="s">
+      <c r="C34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D34" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A35" s="5" t="s">
+      <c r="A35" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="B35" s="5" t="s">
+      <c r="B35" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" s="5" t="s">
+      <c r="C35" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A36" s="5" t="s">
+      <c r="A36" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B36" s="5" t="s">
+      <c r="B36" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C36" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" s="5" t="s">
+      <c r="C36" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A37" s="5" t="s">
+      <c r="A37" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" s="5" t="s">
+      <c r="C37" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A38" s="5" t="s">
+      <c r="A38" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C38" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" s="5" t="s">
+      <c r="C38" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="A39" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B39" t="s">
+      <c r="B39" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C39" t="s">
-        <v>6</v>
-      </c>
-      <c r="D39" t="s">
+      <c r="C39" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="A40" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B40" t="s">
+      <c r="B40" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C40" t="s">
-        <v>11</v>
-      </c>
-      <c r="D40" t="s">
+      <c r="C40" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A41" s="4" t="s">
+      <c r="A41" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B41" s="4" t="s">
+      <c r="B41" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D41" s="4" t="s">
+      <c r="C41" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D41" s="2" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1247,72 +1247,72 @@
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="5" t="s">
+      <c r="A45" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="B45" s="5" t="s">
+      <c r="B45" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="5" t="s">
+      <c r="C45" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D45" s="3" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="5" t="s">
+      <c r="A46" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B46" s="5" t="s">
+      <c r="B46" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C46" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D46" s="5" t="s">
+      <c r="C46" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A47" s="5" t="s">
+      <c r="A47" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B47" s="5" t="s">
+      <c r="B47" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C47" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" s="5" t="s">
+      <c r="C47" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="3" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A48" s="5" t="s">
+      <c r="A48" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B48" s="5" t="s">
+      <c r="B48" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C48" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D48" s="5" t="s">
+      <c r="C48" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A49" s="5" t="s">
+      <c r="A49" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B49" s="5" t="s">
+      <c r="B49" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C49" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" s="5" t="s">
+      <c r="C49" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1346,12 +1346,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">

</xml_diff>

<commit_message>
feat: forms de basicRegistration
</commit_message>
<xml_diff>
--- a/documentacao-e-dados-auxiliares/backlog.xlsx
+++ b/documentacao-e-dados-auxiliares/backlog.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Biblioteca\projetos\sistema-resgistro-analise-integrada\documentacao-e-dados-auxiliares\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{083567BC-7442-443F-A159-8344CCC19DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D216185C-CA59-43E5-8273-5775F50FC894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -258,7 +258,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -279,14 +279,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
-        <bgColor rgb="FFFFCC00"/>
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor rgb="FFFFCC00"/>
       </patternFill>
     </fill>
   </fills>
@@ -302,16 +308,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -995,16 +1002,16 @@
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
+      <c r="A27" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D27" s="5" t="s">
+      <c r="C27" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="7" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1023,16 +1030,16 @@
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="5" t="s">
+      <c r="A29" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D29" s="5" t="s">
+      <c r="C29" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D29" s="7" t="s">
         <v>12</v>
       </c>
     </row>
@@ -1205,44 +1212,44 @@
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="A42" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B42" t="s">
+      <c r="B42" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C42" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" t="s">
+      <c r="C42" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D42" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="A43" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="B43" t="s">
+      <c r="B43" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C43" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" t="s">
+      <c r="C43" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="4" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+      <c r="A44" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C44" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" t="s">
+      <c r="C44" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1322,7 +1329,7 @@
       <formula1>$G$3:$G$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D48:D52 D2:D46" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D48:D52 D2:D26 D27:D46" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>$H$3:$H$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1346,12 +1353,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">

</xml_diff>